<commit_message>
Cargar desde archivo en la ficha del cliente (solo Excel con el formato de la plantilla)
- Valida que sea Excel por contenido; si no, explica y ofrece la plantilla
- Lee plan, datos del cliente y nutrición; vista previa con casillas para elegir qué aplicar
- Asigna el plan y lo programa en el calendario (reemplaza pendientes del plan anterior)
- Plantilla ampliada con hojas «Datos del cliente» y «Nutrición»

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EqTd92FjD8shfoXfrWiS9M
</commit_message>
<xml_diff>
--- a/plantilla-entrenamiento.xlsx
+++ b/plantilla-entrenamiento.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos del plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quads" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hams &amp; Glutes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shoulder &amp; Tricep" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back &amp; Bicep" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chest" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos del cliente" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hams &amp; Glutes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shoulder &amp; Tricep" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back &amp; Bicep" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chest" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrición" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -127,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -174,6 +176,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -539,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -600,7 +612,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>5. Guarda como .xlsx y súbelo en el portal: Panel del coach → Plantillas → «Subir Excel». Se abre el editor para que lo revises antes de guardar.</t>
+          <t>5. Guarda como .xlsx y súbelo en el portal: en la ficha del cliente → «Cargar desde archivo» (se asigna a ese cliente) o en Plantillas → «Cargar desde archivo» (queda como plantilla).</t>
         </is>
       </c>
     </row>
@@ -676,26 +688,57 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>REGLAS</t>
+          <t>HOJAS OPCIONALES (en la ficha del cliente → «Cargar desde archivo»)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>• No cambies ni muevas la fila de encabezados (la que dice Ejercicio).</t>
+          <t>Datos del cliente: edad, género, peso, estatura, % grasa, masa muscular, FC en reposo, nivel de actividad, objetivo, peso meta y kcal del plan. Deja vacío lo que no quieras cambiar.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>• Las filas sin nombre de ejercicio se ignoran. Escribe NA o deja vacío lo que no aplique.</t>
+          <t>Nutrición: una fila por comida con Hora, Comida, Alimentos (separados por coma), kcal y Suplementos. Si no hay plan de alimentación, borra la hoja.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Al cargarlo en la ficha de un cliente, el plan se asigna y se programa en su calendario; también se actualizan su alimentación y sus datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>REGLAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>• No cambies ni muevas la fila de encabezados (la que dice Ejercicio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>• Las filas sin nombre de ejercicio se ignoran. Escribe NA o deja vacío lo que no aplique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>• La hoja «Instrucciones» no se importa.</t>
         </is>
@@ -778,1213 +821,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>QUADS</t>
+          <t>DATOS DEL CLIENTE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Reemplaza los ejercicios de ejemplo. Misma letra en Combinación (filas seguidas) = biserie, triserie o megaserie. No muevas la fila de encabezados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Combinación</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Ejercicio</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>F1 Series</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>F1 Reps</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>F2 Series</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>F2 Reps</t>
-        </is>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>F3 Series</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
-        <is>
-          <t>F3 Reps</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>F4 Series</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>F4 Reps</t>
-        </is>
-      </c>
-      <c r="M3" s="10" t="inlineStr">
-        <is>
-          <t>Tempo</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>RIR</t>
-        </is>
-      </c>
-      <c r="O3" s="10" t="inlineStr">
-        <is>
-          <t>Descanso</t>
-        </is>
-      </c>
-      <c r="P3" s="10" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="Q3" s="10" t="inlineStr">
-        <is>
-          <t>Video</t>
+          <t>Opcional. Deja vacío lo que no quieras cambiar.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr"/>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Aislado</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Extensión de cuádriceps</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="I4" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L4" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M4" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-1</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" s="13" t="inlineStr">
-        <is>
-          <t>60 s</t>
-        </is>
-      </c>
-      <c r="P4" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q4" s="12" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Género</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Mujer u Hombre</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr"/>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Aislado</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Sentadilla trasera</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="I5" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="M5" s="13" t="inlineStr">
-        <is>
-          <t>3-1-1-0</t>
-        </is>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" s="13" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="P5" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Edad</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>años</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Biserie</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Prensa 45°</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I6" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="J6" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="M6" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-0</t>
-        </is>
-      </c>
-      <c r="N6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="13" t="inlineStr"/>
-      <c r="P6" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q6" s="12" t="inlineStr"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Peso (kg)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>Biserie</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Zancada búlgara</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>10 c/p</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>10 c/p</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="14" t="inlineStr">
-        <is>
-          <t>8 c/p</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>8 c/p</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-0</t>
-        </is>
-      </c>
-      <c r="N7" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" s="13" t="inlineStr">
-        <is>
-          <t>90 s</t>
-        </is>
-      </c>
-      <c r="P7" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q7" s="12" t="inlineStr"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Estatura (cm)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>164</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>Triserie</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>Sentadilla goblet</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I8" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M8" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-0</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="13" t="inlineStr"/>
-      <c r="P8" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q8" s="12" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>% grasa</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>Triserie</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Sissy squat</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="I9" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="M9" s="13" t="inlineStr">
-        <is>
-          <t>3-0-1-0</t>
-        </is>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="13" t="inlineStr"/>
-      <c r="P9" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Masa muscular (kg)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>Triserie</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>Extensión unilateral</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I10" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K10" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M10" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-1</t>
-        </is>
-      </c>
-      <c r="N10" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="13" t="inlineStr">
-        <is>
-          <t>90 s</t>
-        </is>
-      </c>
-      <c r="P10" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q10" s="12" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>FC en reposo (lpm)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>para zonas de Karvonen</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr"/>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Dropset</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Prensa unilateral</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K11" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="M11" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-0</t>
-        </is>
-      </c>
-      <c r="N11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="13" t="inlineStr">
-        <is>
-          <t>60 s</t>
-        </is>
-      </c>
-      <c r="P11" s="13" t="inlineStr">
-        <is>
-          <t>lb</t>
-        </is>
-      </c>
-      <c r="Q11" s="12" t="inlineStr"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Nivel de actividad</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Sedentario, Ligero, Moderado, Alto o Muy alto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
-      <c r="M12" s="19" t="n"/>
-      <c r="N12" s="19" t="n"/>
-      <c r="O12" s="19" t="n"/>
-      <c r="P12" s="19" t="n"/>
-      <c r="Q12" s="19" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Hipertrofia</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
-      <c r="I13" s="19" t="n"/>
-      <c r="J13" s="19" t="n"/>
-      <c r="K13" s="19" t="n"/>
-      <c r="L13" s="19" t="n"/>
-      <c r="M13" s="19" t="n"/>
-      <c r="N13" s="19" t="n"/>
-      <c r="O13" s="19" t="n"/>
-      <c r="P13" s="19" t="n"/>
-      <c r="Q13" s="19" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Peso meta (kg)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="19" t="n"/>
-      <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
-      <c r="I14" s="19" t="n"/>
-      <c r="J14" s="19" t="n"/>
-      <c r="K14" s="19" t="n"/>
-      <c r="L14" s="19" t="n"/>
-      <c r="M14" s="19" t="n"/>
-      <c r="N14" s="19" t="n"/>
-      <c r="O14" s="19" t="n"/>
-      <c r="P14" s="19" t="n"/>
-      <c r="Q14" s="19" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="19" t="n"/>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
-      <c r="I15" s="19" t="n"/>
-      <c r="J15" s="19" t="n"/>
-      <c r="K15" s="19" t="n"/>
-      <c r="L15" s="19" t="n"/>
-      <c r="M15" s="19" t="n"/>
-      <c r="N15" s="19" t="n"/>
-      <c r="O15" s="19" t="n"/>
-      <c r="P15" s="19" t="n"/>
-      <c r="Q15" s="19" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="19" t="n"/>
-      <c r="H16" s="19" t="n"/>
-      <c r="I16" s="19" t="n"/>
-      <c r="J16" s="19" t="n"/>
-      <c r="K16" s="19" t="n"/>
-      <c r="L16" s="19" t="n"/>
-      <c r="M16" s="19" t="n"/>
-      <c r="N16" s="19" t="n"/>
-      <c r="O16" s="19" t="n"/>
-      <c r="P16" s="19" t="n"/>
-      <c r="Q16" s="19" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="19" t="n"/>
-      <c r="G17" s="19" t="n"/>
-      <c r="H17" s="19" t="n"/>
-      <c r="I17" s="19" t="n"/>
-      <c r="J17" s="19" t="n"/>
-      <c r="K17" s="19" t="n"/>
-      <c r="L17" s="19" t="n"/>
-      <c r="M17" s="19" t="n"/>
-      <c r="N17" s="19" t="n"/>
-      <c r="O17" s="19" t="n"/>
-      <c r="P17" s="19" t="n"/>
-      <c r="Q17" s="19" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="19" t="n"/>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="19" t="n"/>
-      <c r="G18" s="19" t="n"/>
-      <c r="H18" s="19" t="n"/>
-      <c r="I18" s="19" t="n"/>
-      <c r="J18" s="19" t="n"/>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="19" t="n"/>
-      <c r="M18" s="19" t="n"/>
-      <c r="N18" s="19" t="n"/>
-      <c r="O18" s="19" t="n"/>
-      <c r="P18" s="19" t="n"/>
-      <c r="Q18" s="19" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="19" t="n"/>
-      <c r="G19" s="19" t="n"/>
-      <c r="H19" s="19" t="n"/>
-      <c r="I19" s="19" t="n"/>
-      <c r="J19" s="19" t="n"/>
-      <c r="K19" s="19" t="n"/>
-      <c r="L19" s="19" t="n"/>
-      <c r="M19" s="19" t="n"/>
-      <c r="N19" s="19" t="n"/>
-      <c r="O19" s="19" t="n"/>
-      <c r="P19" s="19" t="n"/>
-      <c r="Q19" s="19" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
-      <c r="I20" s="19" t="n"/>
-      <c r="J20" s="19" t="n"/>
-      <c r="K20" s="19" t="n"/>
-      <c r="L20" s="19" t="n"/>
-      <c r="M20" s="19" t="n"/>
-      <c r="N20" s="19" t="n"/>
-      <c r="O20" s="19" t="n"/>
-      <c r="P20" s="19" t="n"/>
-      <c r="Q20" s="19" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="19" t="n"/>
-      <c r="G21" s="19" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="19" t="n"/>
-      <c r="J21" s="19" t="n"/>
-      <c r="K21" s="19" t="n"/>
-      <c r="L21" s="19" t="n"/>
-      <c r="M21" s="19" t="n"/>
-      <c r="N21" s="19" t="n"/>
-      <c r="O21" s="19" t="n"/>
-      <c r="P21" s="19" t="n"/>
-      <c r="Q21" s="19" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="19" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
-      <c r="M22" s="19" t="n"/>
-      <c r="N22" s="19" t="n"/>
-      <c r="O22" s="19" t="n"/>
-      <c r="P22" s="19" t="n"/>
-      <c r="Q22" s="19" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
-      <c r="H23" s="19" t="n"/>
-      <c r="I23" s="19" t="n"/>
-      <c r="J23" s="19" t="n"/>
-      <c r="K23" s="19" t="n"/>
-      <c r="L23" s="19" t="n"/>
-      <c r="M23" s="19" t="n"/>
-      <c r="N23" s="19" t="n"/>
-      <c r="O23" s="19" t="n"/>
-      <c r="P23" s="19" t="n"/>
-      <c r="Q23" s="19" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-      <c r="G24" s="19" t="n"/>
-      <c r="H24" s="19" t="n"/>
-      <c r="I24" s="19" t="n"/>
-      <c r="J24" s="19" t="n"/>
-      <c r="K24" s="19" t="n"/>
-      <c r="L24" s="19" t="n"/>
-      <c r="M24" s="19" t="n"/>
-      <c r="N24" s="19" t="n"/>
-      <c r="O24" s="19" t="n"/>
-      <c r="P24" s="19" t="n"/>
-      <c r="Q24" s="19" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="19" t="n"/>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="19" t="n"/>
-      <c r="F25" s="19" t="n"/>
-      <c r="G25" s="19" t="n"/>
-      <c r="H25" s="19" t="n"/>
-      <c r="I25" s="19" t="n"/>
-      <c r="J25" s="19" t="n"/>
-      <c r="K25" s="19" t="n"/>
-      <c r="L25" s="19" t="n"/>
-      <c r="M25" s="19" t="n"/>
-      <c r="N25" s="19" t="n"/>
-      <c r="O25" s="19" t="n"/>
-      <c r="P25" s="19" t="n"/>
-      <c r="Q25" s="19" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="19" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
-      <c r="G26" s="19" t="n"/>
-      <c r="H26" s="19" t="n"/>
-      <c r="I26" s="19" t="n"/>
-      <c r="J26" s="19" t="n"/>
-      <c r="K26" s="19" t="n"/>
-      <c r="L26" s="19" t="n"/>
-      <c r="M26" s="19" t="n"/>
-      <c r="N26" s="19" t="n"/>
-      <c r="O26" s="19" t="n"/>
-      <c r="P26" s="19" t="n"/>
-      <c r="Q26" s="19" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="19" t="n"/>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
-      <c r="G27" s="19" t="n"/>
-      <c r="H27" s="19" t="n"/>
-      <c r="I27" s="19" t="n"/>
-      <c r="J27" s="19" t="n"/>
-      <c r="K27" s="19" t="n"/>
-      <c r="L27" s="19" t="n"/>
-      <c r="M27" s="19" t="n"/>
-      <c r="N27" s="19" t="n"/>
-      <c r="O27" s="19" t="n"/>
-      <c r="P27" s="19" t="n"/>
-      <c r="Q27" s="19" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="19" t="n"/>
-      <c r="G28" s="19" t="n"/>
-      <c r="H28" s="19" t="n"/>
-      <c r="I28" s="19" t="n"/>
-      <c r="J28" s="19" t="n"/>
-      <c r="K28" s="19" t="n"/>
-      <c r="L28" s="19" t="n"/>
-      <c r="M28" s="19" t="n"/>
-      <c r="N28" s="19" t="n"/>
-      <c r="O28" s="19" t="n"/>
-      <c r="P28" s="19" t="n"/>
-      <c r="Q28" s="19" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="19" t="n"/>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="19" t="n"/>
-      <c r="F29" s="19" t="n"/>
-      <c r="G29" s="19" t="n"/>
-      <c r="H29" s="19" t="n"/>
-      <c r="I29" s="19" t="n"/>
-      <c r="J29" s="19" t="n"/>
-      <c r="K29" s="19" t="n"/>
-      <c r="L29" s="19" t="n"/>
-      <c r="M29" s="19" t="n"/>
-      <c r="N29" s="19" t="n"/>
-      <c r="O29" s="19" t="n"/>
-      <c r="P29" s="19" t="n"/>
-      <c r="Q29" s="19" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="19" t="n"/>
-      <c r="F30" s="19" t="n"/>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="19" t="n"/>
-      <c r="J30" s="19" t="n"/>
-      <c r="K30" s="19" t="n"/>
-      <c r="L30" s="19" t="n"/>
-      <c r="M30" s="19" t="n"/>
-      <c r="N30" s="19" t="n"/>
-      <c r="O30" s="19" t="n"/>
-      <c r="P30" s="19" t="n"/>
-      <c r="Q30" s="19" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="19" t="n"/>
-      <c r="F31" s="19" t="n"/>
-      <c r="G31" s="19" t="n"/>
-      <c r="H31" s="19" t="n"/>
-      <c r="I31" s="19" t="n"/>
-      <c r="J31" s="19" t="n"/>
-      <c r="K31" s="19" t="n"/>
-      <c r="L31" s="19" t="n"/>
-      <c r="M31" s="19" t="n"/>
-      <c r="N31" s="19" t="n"/>
-      <c r="O31" s="19" t="n"/>
-      <c r="P31" s="19" t="n"/>
-      <c r="Q31" s="19" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="19" t="n"/>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="19" t="n"/>
-      <c r="F32" s="19" t="n"/>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="19" t="n"/>
-      <c r="J32" s="19" t="n"/>
-      <c r="K32" s="19" t="n"/>
-      <c r="L32" s="19" t="n"/>
-      <c r="M32" s="19" t="n"/>
-      <c r="N32" s="19" t="n"/>
-      <c r="O32" s="19" t="n"/>
-      <c r="P32" s="19" t="n"/>
-      <c r="Q32" s="19" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
-      <c r="F33" s="19" t="n"/>
-      <c r="G33" s="19" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="19" t="n"/>
-      <c r="J33" s="19" t="n"/>
-      <c r="K33" s="19" t="n"/>
-      <c r="L33" s="19" t="n"/>
-      <c r="M33" s="19" t="n"/>
-      <c r="N33" s="19" t="n"/>
-      <c r="O33" s="19" t="n"/>
-      <c r="P33" s="19" t="n"/>
-      <c r="Q33" s="19" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="19" t="n"/>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="19" t="n"/>
-      <c r="F34" s="19" t="n"/>
-      <c r="G34" s="19" t="n"/>
-      <c r="H34" s="19" t="n"/>
-      <c r="I34" s="19" t="n"/>
-      <c r="J34" s="19" t="n"/>
-      <c r="K34" s="19" t="n"/>
-      <c r="L34" s="19" t="n"/>
-      <c r="M34" s="19" t="n"/>
-      <c r="N34" s="19" t="n"/>
-      <c r="O34" s="19" t="n"/>
-      <c r="P34" s="19" t="n"/>
-      <c r="Q34" s="19" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="19" t="n"/>
-      <c r="B35" s="19" t="n"/>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
-      <c r="G35" s="19" t="n"/>
-      <c r="H35" s="19" t="n"/>
-      <c r="I35" s="19" t="n"/>
-      <c r="J35" s="19" t="n"/>
-      <c r="K35" s="19" t="n"/>
-      <c r="L35" s="19" t="n"/>
-      <c r="M35" s="19" t="n"/>
-      <c r="N35" s="19" t="n"/>
-      <c r="O35" s="19" t="n"/>
-      <c r="P35" s="19" t="n"/>
-      <c r="Q35" s="19" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="19" t="n"/>
-      <c r="B36" s="19" t="n"/>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="19" t="n"/>
-      <c r="F36" s="19" t="n"/>
-      <c r="G36" s="19" t="n"/>
-      <c r="H36" s="19" t="n"/>
-      <c r="I36" s="19" t="n"/>
-      <c r="J36" s="19" t="n"/>
-      <c r="K36" s="19" t="n"/>
-      <c r="L36" s="19" t="n"/>
-      <c r="M36" s="19" t="n"/>
-      <c r="N36" s="19" t="n"/>
-      <c r="O36" s="19" t="n"/>
-      <c r="P36" s="19" t="n"/>
-      <c r="Q36" s="19" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="n"/>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
-      <c r="F37" s="19" t="n"/>
-      <c r="G37" s="19" t="n"/>
-      <c r="H37" s="19" t="n"/>
-      <c r="I37" s="19" t="n"/>
-      <c r="J37" s="19" t="n"/>
-      <c r="K37" s="19" t="n"/>
-      <c r="L37" s="19" t="n"/>
-      <c r="M37" s="19" t="n"/>
-      <c r="N37" s="19" t="n"/>
-      <c r="O37" s="19" t="n"/>
-      <c r="P37" s="19" t="n"/>
-      <c r="Q37" s="19" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="n"/>
-      <c r="B38" s="19" t="n"/>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="19" t="n"/>
-      <c r="E38" s="19" t="n"/>
-      <c r="F38" s="19" t="n"/>
-      <c r="G38" s="19" t="n"/>
-      <c r="H38" s="19" t="n"/>
-      <c r="I38" s="19" t="n"/>
-      <c r="J38" s="19" t="n"/>
-      <c r="K38" s="19" t="n"/>
-      <c r="L38" s="19" t="n"/>
-      <c r="M38" s="19" t="n"/>
-      <c r="N38" s="19" t="n"/>
-      <c r="O38" s="19" t="n"/>
-      <c r="P38" s="19" t="n"/>
-      <c r="Q38" s="19" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="19" t="n"/>
-      <c r="B39" s="19" t="n"/>
-      <c r="C39" s="19" t="n"/>
-      <c r="D39" s="19" t="n"/>
-      <c r="E39" s="19" t="n"/>
-      <c r="F39" s="19" t="n"/>
-      <c r="G39" s="19" t="n"/>
-      <c r="H39" s="19" t="n"/>
-      <c r="I39" s="19" t="n"/>
-      <c r="J39" s="19" t="n"/>
-      <c r="K39" s="19" t="n"/>
-      <c r="L39" s="19" t="n"/>
-      <c r="M39" s="19" t="n"/>
-      <c r="N39" s="19" t="n"/>
-      <c r="O39" s="19" t="n"/>
-      <c r="P39" s="19" t="n"/>
-      <c r="Q39" s="19" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="I40" s="19" t="n"/>
-      <c r="J40" s="19" t="n"/>
-      <c r="K40" s="19" t="n"/>
-      <c r="L40" s="19" t="n"/>
-      <c r="M40" s="19" t="n"/>
-      <c r="N40" s="19" t="n"/>
-      <c r="O40" s="19" t="n"/>
-      <c r="P40" s="19" t="n"/>
-      <c r="Q40" s="19" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Kcal del plan</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>kcal/día</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mujer,Hombre"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
-    </dataValidation>
-    <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"kg,lb"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B4:B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"A,B,C,D,E,F,G,H"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E4:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="G4:G40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="I4:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
-    </dataValidation>
-    <dataValidation sqref="K4:K40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>20</formula2>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sedentario,Ligero,Moderado,Alto,Muy alto"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2022,7 +1034,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>HAMS &amp; GLUTES</t>
+          <t>QUADS</t>
         </is>
       </c>
     </row>
@@ -2134,44 +1146,36 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Hip thrust con barra</t>
+          <t>Extensión de cuádriceps</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>8-10</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>15</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>8-10</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>15</v>
       </c>
       <c r="I4" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>6-8</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>12</v>
       </c>
       <c r="K4" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>6-8</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <v>12</v>
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>2-1-1-1</t>
+          <t>2-0-1-1</t>
         </is>
       </c>
       <c r="N4" s="13" t="n">
@@ -2179,7 +1183,7 @@
       </c>
       <c r="O4" s="13" t="inlineStr">
         <is>
-          <t>90 s</t>
+          <t>60 s</t>
         </is>
       </c>
       <c r="P4" s="13" t="inlineStr">
@@ -2203,7 +1207,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Peso muerto rumano</t>
+          <t>Sentadilla trasera</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
@@ -2219,20 +1223,20 @@
         <v>8</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J5" s="14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L5" s="13" t="n">
         <v>6</v>
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>3-0-1-0</t>
+          <t>3-1-1-0</t>
         </is>
       </c>
       <c r="N5" s="13" t="n">
@@ -2263,12 +1267,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Superserie</t>
+          <t>Biserie</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Curl femoral acostado</t>
+          <t>Prensa 45°</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
@@ -2284,24 +1288,24 @@
         <v>12</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="14" t="n">
         <v>10</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="13" t="n">
         <v>10</v>
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N6" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="13" t="inlineStr"/>
       <c r="P6" s="13" t="inlineStr">
@@ -2324,49 +1328,57 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Superserie</t>
+          <t>Biserie</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Extensión de cadera en polea</t>
+          <t>Zancada búlgara</t>
         </is>
       </c>
       <c r="E7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="14" t="n">
-        <v>15</v>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>10 c/p</t>
+        </is>
       </c>
       <c r="G7" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="13" t="n">
-        <v>15</v>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>10 c/p</t>
+        </is>
       </c>
       <c r="I7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="14" t="n">
-        <v>12</v>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>8 c/p</t>
+        </is>
       </c>
       <c r="K7" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="13" t="n">
-        <v>12</v>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>8 c/p</t>
+        </is>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N7" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>60 s</t>
+          <t>90 s</t>
         </is>
       </c>
       <c r="P7" s="13" t="inlineStr">
@@ -2382,117 +1394,247 @@
           <t>Complementario</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr"/>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Dropset</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Abducción en máquina</t>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Triserie</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Sentadilla goblet</t>
         </is>
       </c>
       <c r="E8" s="14" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>3</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I8" s="14" t="n">
         <v>3</v>
       </c>
       <c r="J8" s="14" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K8" s="13" t="n">
         <v>3</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N8" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q8" s="12" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Triserie</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Sissy squat</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>3-0-1-0</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="13" t="inlineStr"/>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Triserie</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Extensión unilateral</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-1</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>90 s</t>
+        </is>
+      </c>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr"/>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Dropset</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Prensa unilateral</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-0</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
         <is>
           <t>60 s</t>
         </is>
       </c>
-      <c r="P8" s="13" t="inlineStr">
+      <c r="P11" s="13" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="19" t="n"/>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="19" t="n"/>
-      <c r="J9" s="19" t="n"/>
-      <c r="K9" s="19" t="n"/>
-      <c r="L9" s="19" t="n"/>
-      <c r="M9" s="19" t="n"/>
-      <c r="N9" s="19" t="n"/>
-      <c r="O9" s="19" t="n"/>
-      <c r="P9" s="19" t="n"/>
-      <c r="Q9" s="19" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="19" t="n"/>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="19" t="n"/>
-      <c r="O10" s="19" t="n"/>
-      <c r="P10" s="19" t="n"/>
-      <c r="Q10" s="19" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
-      <c r="I11" s="19" t="n"/>
-      <c r="J11" s="19" t="n"/>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="19" t="n"/>
-      <c r="M11" s="19" t="n"/>
-      <c r="N11" s="19" t="n"/>
-      <c r="O11" s="19" t="n"/>
-      <c r="P11" s="19" t="n"/>
-      <c r="Q11" s="19" t="n"/>
+      <c r="Q11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n"/>
@@ -3111,7 +2253,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>SHOULDER &amp; TRICEP</t>
+          <t>HAMS &amp; GLUTES</t>
         </is>
       </c>
     </row>
@@ -3223,44 +2365,52 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Elevaciones laterales</t>
+          <t>Hip thrust con barra</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="14" t="n">
-        <v>12</v>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>8-10</t>
+        </is>
       </c>
       <c r="G4" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="13" t="n">
-        <v>12</v>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>8-10</t>
+        </is>
       </c>
       <c r="I4" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="J4" s="14" t="n">
-        <v>12</v>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
       </c>
       <c r="K4" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="L4" s="13" t="n">
-        <v>12</v>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-1-1-1</t>
         </is>
       </c>
       <c r="N4" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="13" t="inlineStr">
         <is>
-          <t>60 s</t>
+          <t>90 s</t>
         </is>
       </c>
       <c r="P4" s="13" t="inlineStr">
@@ -3284,7 +2434,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Press militar con mancuernas</t>
+          <t>Peso muerto rumano</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
@@ -3313,7 +2463,7 @@
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-0</t>
+          <t>3-0-1-0</t>
         </is>
       </c>
       <c r="N5" s="13" t="n">
@@ -3321,7 +2471,7 @@
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>90 s</t>
+          <t>2 min</t>
         </is>
       </c>
       <c r="P5" s="13" t="inlineStr">
@@ -3334,7 +2484,7 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Complementario</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -3344,12 +2494,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Biserie</t>
+          <t>Superserie</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Fondos en máquina</t>
+          <t>Curl femoral acostado</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
@@ -3378,7 +2528,7 @@
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-0</t>
+          <t>2-0-1-1</t>
         </is>
       </c>
       <c r="N6" s="13" t="n">
@@ -3395,7 +2545,7 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Complementario</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -3405,25 +2555,25 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Biserie</t>
+          <t>Superserie</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Extensión de tríceps en polea</t>
+          <t>Extensión de cadera en polea</t>
         </is>
       </c>
       <c r="E7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>3</v>
@@ -3458,23 +2608,65 @@
       <c r="Q7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="19" t="n"/>
-      <c r="J8" s="19" t="n"/>
-      <c r="K8" s="19" t="n"/>
-      <c r="L8" s="19" t="n"/>
-      <c r="M8" s="19" t="n"/>
-      <c r="N8" s="19" t="n"/>
-      <c r="O8" s="19" t="n"/>
-      <c r="P8" s="19" t="n"/>
-      <c r="Q8" s="19" t="n"/>
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr"/>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Dropset</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Abducción en máquina</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>60 s</t>
+        </is>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>lb</t>
+        </is>
+      </c>
+      <c r="Q8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="n"/>
@@ -4150,7 +3342,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>BACK &amp; BICEP</t>
+          <t>SHOULDER &amp; TRICEP</t>
         </is>
       </c>
     </row>
@@ -4262,32 +3454,32 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Face pull</t>
+          <t>Elevaciones laterales</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I4" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="14" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K4" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" s="13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
@@ -4323,7 +3515,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Jalón al pecho</t>
+          <t>Press militar con mancuernas</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
@@ -4336,7 +3528,7 @@
         <v>4</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I5" s="14" t="n">
         <v>4</v>
@@ -4348,11 +3540,11 @@
         <v>4</v>
       </c>
       <c r="L5" s="13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N5" s="13" t="n">
@@ -4373,57 +3565,57 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr"/>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Aislado</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Remo con mancuerna</t>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Biserie</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Fondos en máquina</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="13" t="n">
+      <c r="K6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="I6" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="J6" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K6" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="13" t="n">
-        <v>8</v>
-      </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="13" t="inlineStr">
-        <is>
-          <t>90 s</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O6" s="13" t="inlineStr"/>
       <c r="P6" s="13" t="inlineStr">
         <is>
           <t>kg</t>
@@ -4444,47 +3636,51 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Superserie</t>
+          <t>Biserie</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Curl con barra</t>
+          <t>Extensión de tríceps en polea</t>
         </is>
       </c>
       <c r="E7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-0</t>
+          <t>2-0-1-1</t>
         </is>
       </c>
       <c r="N7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="13" t="inlineStr"/>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>60 s</t>
+        </is>
+      </c>
       <c r="P7" s="13" t="inlineStr">
         <is>
           <t>kg</t>
@@ -4493,69 +3689,23 @@
       <c r="Q7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Superserie</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Curl martillo</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I8" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="M8" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-0</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="13" t="inlineStr">
-        <is>
-          <t>60 s</t>
-        </is>
-      </c>
-      <c r="P8" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q8" s="12" t="inlineStr"/>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="19" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="19" t="n"/>
+      <c r="P8" s="19" t="n"/>
+      <c r="Q8" s="19" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="n"/>
@@ -5231,7 +4381,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>CHEST</t>
+          <t>BACK &amp; BICEP</t>
         </is>
       </c>
     </row>
@@ -5343,7 +4493,7 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Aperturas en peck deck</t>
+          <t>Face pull</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
@@ -5362,13 +4512,13 @@
         <v>3</v>
       </c>
       <c r="J4" s="14" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K4" s="13" t="n">
         <v>3</v>
       </c>
       <c r="L4" s="13" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
@@ -5376,7 +4526,7 @@
         </is>
       </c>
       <c r="N4" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" s="13" t="inlineStr">
         <is>
@@ -5404,7 +4554,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Press de banca</t>
+          <t>Jalón al pecho</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
@@ -5417,23 +4567,23 @@
         <v>4</v>
       </c>
       <c r="H5" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>6</v>
-      </c>
       <c r="K5" s="13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L5" s="13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>3-1-1-0</t>
+          <t>2-0-1-1</t>
         </is>
       </c>
       <c r="N5" s="13" t="n">
@@ -5441,7 +4591,7 @@
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>90 s</t>
         </is>
       </c>
       <c r="P5" s="13" t="inlineStr">
@@ -5454,57 +4604,57 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Megaserie</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Press inclinado con mancuernas</t>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr"/>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Aislado</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Remo con mancuerna</t>
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="14" t="n">
         <v>10</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H6" s="13" t="n">
         <v>10</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-0</t>
+          <t>2-0-1-1</t>
         </is>
       </c>
       <c r="N6" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>90 s</t>
+        </is>
+      </c>
       <c r="P6" s="13" t="inlineStr">
         <is>
           <t>kg</t>
@@ -5525,41 +4675,41 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Megaserie</t>
+          <t>Superserie</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Cruce de poleas</t>
+          <t>Curl con barra</t>
         </is>
       </c>
       <c r="E7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K7" s="13" t="n">
         <v>3</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>2-0-1-1</t>
+          <t>2-0-1-0</t>
         </is>
       </c>
       <c r="N7" s="13" t="n">
@@ -5586,57 +4736,51 @@
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Megaserie</t>
+          <t>Superserie</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Lagartijas</t>
+          <t>Curl martillo</t>
         </is>
       </c>
       <c r="E8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>AMRAP</t>
-        </is>
+      <c r="F8" s="14" t="n">
+        <v>12</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>AMRAP</t>
-        </is>
+      <c r="H8" s="13" t="n">
+        <v>12</v>
       </c>
       <c r="I8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>AMRAP</t>
-        </is>
+      <c r="J8" s="14" t="n">
+        <v>10</v>
       </c>
       <c r="K8" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>AMRAP</t>
-        </is>
+      <c r="L8" s="13" t="n">
+        <v>10</v>
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="O8" s="13" t="inlineStr"/>
+          <t>2-0-1-0</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="13" t="inlineStr">
+        <is>
+          <t>60 s</t>
+        </is>
+      </c>
       <c r="P8" s="13" t="inlineStr">
         <is>
           <t>kg</t>
@@ -5645,69 +4789,23 @@
       <c r="Q8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Megaserie</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Pullover en polea</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I9" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" s="13" t="inlineStr">
-        <is>
-          <t>2-0-1-1</t>
-        </is>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="13" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="P9" s="13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr"/>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="19" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="19" t="n"/>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="19" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="19" t="n"/>
+      <c r="O9" s="19" t="n"/>
+      <c r="P9" s="19" t="n"/>
+      <c r="Q9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="n"/>
@@ -6331,4 +5429,1440 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>CHEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Reemplaza los ejercicios de ejemplo. Misma letra en Combinación (filas seguidas) = biserie, triserie o megaserie. No muevas la fila de encabezados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Combinación</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Ejercicio</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>F1 Series</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>F1 Reps</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>F2 Series</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>F2 Reps</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>F3 Series</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>F3 Reps</t>
+        </is>
+      </c>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>F4 Series</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>F4 Reps</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>RIR</t>
+        </is>
+      </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>Descanso</t>
+        </is>
+      </c>
+      <c r="P3" s="10" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr"/>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Aislado</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Aperturas en peck deck</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-1</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>60 s</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q4" s="12" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr"/>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Aislado</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Press de banca</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>3-1-1-0</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>2 min</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Megaserie</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Press inclinado con mancuernas</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-0</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="13" t="inlineStr"/>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Megaserie</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Cruce de poleas</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-1</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="13" t="inlineStr"/>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Megaserie</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Lagartijas</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>AMRAP</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>AMRAP</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>AMRAP</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>AMRAP</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q8" s="12" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Complementario</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Megaserie</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Pullover en polea</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>2-0-1-1</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>2 min</t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="19" t="n"/>
+      <c r="N10" s="19" t="n"/>
+      <c r="O10" s="19" t="n"/>
+      <c r="P10" s="19" t="n"/>
+      <c r="Q10" s="19" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="19" t="n"/>
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
+      <c r="M11" s="19" t="n"/>
+      <c r="N11" s="19" t="n"/>
+      <c r="O11" s="19" t="n"/>
+      <c r="P11" s="19" t="n"/>
+      <c r="Q11" s="19" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+      <c r="H12" s="19" t="n"/>
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="19" t="n"/>
+      <c r="O12" s="19" t="n"/>
+      <c r="P12" s="19" t="n"/>
+      <c r="Q12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="n"/>
+      <c r="O13" s="19" t="n"/>
+      <c r="P13" s="19" t="n"/>
+      <c r="Q13" s="19" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="19" t="n"/>
+      <c r="N14" s="19" t="n"/>
+      <c r="O14" s="19" t="n"/>
+      <c r="P14" s="19" t="n"/>
+      <c r="Q14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="19" t="n"/>
+      <c r="O15" s="19" t="n"/>
+      <c r="P15" s="19" t="n"/>
+      <c r="Q15" s="19" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="19" t="n"/>
+      <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="19" t="n"/>
+      <c r="L17" s="19" t="n"/>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="n"/>
+      <c r="O17" s="19" t="n"/>
+      <c r="P17" s="19" t="n"/>
+      <c r="Q17" s="19" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="19" t="n"/>
+      <c r="O18" s="19" t="n"/>
+      <c r="P18" s="19" t="n"/>
+      <c r="Q18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
+      <c r="H19" s="19" t="n"/>
+      <c r="I19" s="19" t="n"/>
+      <c r="J19" s="19" t="n"/>
+      <c r="K19" s="19" t="n"/>
+      <c r="L19" s="19" t="n"/>
+      <c r="M19" s="19" t="n"/>
+      <c r="N19" s="19" t="n"/>
+      <c r="O19" s="19" t="n"/>
+      <c r="P19" s="19" t="n"/>
+      <c r="Q19" s="19" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19" t="n"/>
+      <c r="I20" s="19" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="19" t="n"/>
+      <c r="M20" s="19" t="n"/>
+      <c r="N20" s="19" t="n"/>
+      <c r="O20" s="19" t="n"/>
+      <c r="P20" s="19" t="n"/>
+      <c r="Q20" s="19" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="19" t="n"/>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="19" t="n"/>
+      <c r="O21" s="19" t="n"/>
+      <c r="P21" s="19" t="n"/>
+      <c r="Q21" s="19" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
+      <c r="I22" s="19" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="n"/>
+      <c r="O22" s="19" t="n"/>
+      <c r="P22" s="19" t="n"/>
+      <c r="Q22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+      <c r="P23" s="19" t="n"/>
+      <c r="Q23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
+      <c r="I24" s="19" t="n"/>
+      <c r="J24" s="19" t="n"/>
+      <c r="K24" s="19" t="n"/>
+      <c r="L24" s="19" t="n"/>
+      <c r="M24" s="19" t="n"/>
+      <c r="N24" s="19" t="n"/>
+      <c r="O24" s="19" t="n"/>
+      <c r="P24" s="19" t="n"/>
+      <c r="Q24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="19" t="n"/>
+      <c r="K25" s="19" t="n"/>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="19" t="n"/>
+      <c r="O25" s="19" t="n"/>
+      <c r="P25" s="19" t="n"/>
+      <c r="Q25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19" t="n"/>
+      <c r="M26" s="19" t="n"/>
+      <c r="N26" s="19" t="n"/>
+      <c r="O26" s="19" t="n"/>
+      <c r="P26" s="19" t="n"/>
+      <c r="Q26" s="19" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="19" t="n"/>
+      <c r="I27" s="19" t="n"/>
+      <c r="J27" s="19" t="n"/>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="19" t="n"/>
+      <c r="O27" s="19" t="n"/>
+      <c r="P27" s="19" t="n"/>
+      <c r="Q27" s="19" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19" t="n"/>
+      <c r="M28" s="19" t="n"/>
+      <c r="N28" s="19" t="n"/>
+      <c r="O28" s="19" t="n"/>
+      <c r="P28" s="19" t="n"/>
+      <c r="Q28" s="19" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="19" t="n"/>
+      <c r="I29" s="19" t="n"/>
+      <c r="J29" s="19" t="n"/>
+      <c r="K29" s="19" t="n"/>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="19" t="n"/>
+      <c r="O29" s="19" t="n"/>
+      <c r="P29" s="19" t="n"/>
+      <c r="Q29" s="19" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+      <c r="O30" s="19" t="n"/>
+      <c r="P30" s="19" t="n"/>
+      <c r="Q30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="19" t="n"/>
+      <c r="O31" s="19" t="n"/>
+      <c r="P31" s="19" t="n"/>
+      <c r="Q31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="n"/>
+      <c r="H32" s="19" t="n"/>
+      <c r="I32" s="19" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19" t="n"/>
+      <c r="M32" s="19" t="n"/>
+      <c r="N32" s="19" t="n"/>
+      <c r="O32" s="19" t="n"/>
+      <c r="P32" s="19" t="n"/>
+      <c r="Q32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="19" t="n"/>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n"/>
+      <c r="N33" s="19" t="n"/>
+      <c r="O33" s="19" t="n"/>
+      <c r="P33" s="19" t="n"/>
+      <c r="Q33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="n"/>
+      <c r="H34" s="19" t="n"/>
+      <c r="I34" s="19" t="n"/>
+      <c r="J34" s="19" t="n"/>
+      <c r="K34" s="19" t="n"/>
+      <c r="L34" s="19" t="n"/>
+      <c r="M34" s="19" t="n"/>
+      <c r="N34" s="19" t="n"/>
+      <c r="O34" s="19" t="n"/>
+      <c r="P34" s="19" t="n"/>
+      <c r="Q34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="n"/>
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="19" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="19" t="n"/>
+      <c r="O35" s="19" t="n"/>
+      <c r="P35" s="19" t="n"/>
+      <c r="Q35" s="19" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="n"/>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="n"/>
+      <c r="M36" s="19" t="n"/>
+      <c r="N36" s="19" t="n"/>
+      <c r="O36" s="19" t="n"/>
+      <c r="P36" s="19" t="n"/>
+      <c r="Q36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="n"/>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
+      <c r="I37" s="19" t="n"/>
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="19" t="n"/>
+      <c r="N37" s="19" t="n"/>
+      <c r="O37" s="19" t="n"/>
+      <c r="P37" s="19" t="n"/>
+      <c r="Q37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="19" t="n"/>
+      <c r="H38" s="19" t="n"/>
+      <c r="I38" s="19" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="19" t="n"/>
+      <c r="M38" s="19" t="n"/>
+      <c r="N38" s="19" t="n"/>
+      <c r="O38" s="19" t="n"/>
+      <c r="P38" s="19" t="n"/>
+      <c r="Q38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="19" t="n"/>
+      <c r="Q39" s="19" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="n"/>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="19" t="n"/>
+      <c r="I40" s="19" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="19" t="n"/>
+      <c r="L40" s="19" t="n"/>
+      <c r="M40" s="19" t="n"/>
+      <c r="N40" s="19" t="n"/>
+      <c r="O40" s="19" t="n"/>
+      <c r="P40" s="19" t="n"/>
+      <c r="Q40" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="8">
+    <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Rezagado,Principal,Complementario"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"kg,lb"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4:B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B,C,D,E,F,G,H"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="G4:G40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="I4:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="K4:K40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Series" error="Escribe un número entero de series." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>PLAN DE ALIMENTACIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Una fila por comida. Alimentos separados por coma. Si no hay plan de alimentación, borra esta hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Alimentos</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>kcal</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>Suplementos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>7:00</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Desayuno</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Avena 60 g, 3 claras + 1 huevo, 1 plátano</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>520</v>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Creatina 5 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Colación</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Yogur griego 200 g, nueces 20 g, fresas</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>330</v>
+      </c>
+      <c r="E5" s="21" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Arroz 150 g cocido, pechuga 150 g, verduras, aguacate 40 g</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>620</v>
+      </c>
+      <c r="E6" s="21" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Pre-entreno</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Licuado: proteína 1 scoop, leche light, avena 30 g</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>320</v>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>Whey 25 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Cena</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Tortillas de maíz 2, carne magra 120 g, ensalada</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>410</v>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>Magnesio</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="19" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Toma 2.5–3 L de agua al día.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Trabajo aeróbico: máquina, tiempo, inclinación, zona Karvonen y FCE
- Categoría Aeróbico / cardio en el plan y bloque aeróbico en la sesión
- Cambia series/reps/RIR/tempo/descanso por máquina, minutos, inclinación (solo caminadora),
  zona Z1–Z5 y FCE en lpm calculada con Karvonen del cliente
- Vista del atleta con 🏃 y botón «Hecho»; ayuda (?) de FCE
- Excel: columnas Máquina e Inclinación; minutos/zona por fase

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EqTd92FjD8shfoXfrWiS9M
</commit_message>
<xml_diff>
--- a/plantilla-entrenamiento.xlsx
+++ b/plantilla-entrenamiento.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -678,67 +678,74 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Aeróbico: pon Grupo = Aeróbico. En F1–F4 Series escribe los MINUTOS y en F1–F4 Reps la ZONA (Z1 a Z5). Llena Máquina e Inclinación (solo caminadora, en %). La FCE en pulsaciones se calcula sola con la edad y la FC en reposo del cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Video: link de YouTube, Vimeo o Instagram (opcional). Los videos se guardan en tu biblioteca.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>HOJAS OPCIONALES (en la ficha del cliente → «Cargar desde archivo»)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Datos del cliente: edad, género, peso, estatura, % grasa, masa muscular, FC en reposo, nivel de actividad, objetivo, peso meta y kcal del plan. Deja vacío lo que no quieras cambiar.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Nutrición: una fila por comida con Hora, Comida, Alimentos (separados por coma), kcal y Suplementos. Si no hay plan de alimentación, borra la hoja.</t>
+          <t>Datos del cliente: edad, género, peso, estatura, % grasa, masa muscular, FC en reposo, nivel de actividad, objetivo, peso meta y kcal del plan. Deja vacío lo que no quieras cambiar.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>Nutrición: una fila por comida con Hora, Comida, Alimentos (separados por coma), kcal y Suplementos. Si no hay plan de alimentación, borra la hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>Al cargarlo en la ficha de un cliente, el plan se asigna y se programa en su calendario; también se actualizan su alimentación y sus datos.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>REGLAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>• No cambies ni muevas la fila de encabezados (la que dice Ejercicio).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>• Las filas sin nombre de ejercicio se ignoran. Escribe NA o deja vacío lo que no aplique.</t>
+          <t>• No cambies ni muevas la fila de encabezados (la que dice Ejercicio).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>• Las filas sin nombre de ejercicio se ignoran. Escribe NA o deja vacío lo que no aplique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>• La hoja «Instrucciones» no se importa.</t>
         </is>
@@ -1009,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1029,6 +1036,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1131,6 +1140,16 @@
           <t>Video</t>
         </is>
       </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Inclinación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1192,6 +1211,8 @@
         </is>
       </c>
       <c r="Q4" s="12" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
+      <c r="S4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -1253,6 +1274,8 @@
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr"/>
+      <c r="R5" s="13" t="inlineStr"/>
+      <c r="S5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -1314,6 +1337,8 @@
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -1387,6 +1412,8 @@
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -1448,6 +1475,8 @@
         </is>
       </c>
       <c r="Q8" s="12" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
+      <c r="S8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1509,6 +1538,8 @@
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr"/>
+      <c r="R9" s="13" t="inlineStr"/>
+      <c r="S9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -1574,6 +1605,8 @@
         </is>
       </c>
       <c r="Q10" s="12" t="inlineStr"/>
+      <c r="R10" s="13" t="inlineStr"/>
+      <c r="S10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1635,25 +1668,75 @@
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr"/>
+      <c r="R11" s="13" t="inlineStr"/>
+      <c r="S11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
-      <c r="M12" s="19" t="n"/>
-      <c r="N12" s="19" t="n"/>
-      <c r="O12" s="19" t="n"/>
-      <c r="P12" s="19" t="n"/>
-      <c r="Q12" s="19" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Aeróbico</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr"/>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Aeróbico</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Caminata inclinada</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr"/>
+      <c r="N12" s="13" t="inlineStr"/>
+      <c r="O12" s="13" t="inlineStr"/>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q12" s="12" t="inlineStr"/>
+      <c r="R12" s="13" t="inlineStr">
+        <is>
+          <t>Caminadora</t>
+        </is>
+      </c>
+      <c r="S12" s="13" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n"/>
@@ -1673,6 +1756,8 @@
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
       <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n"/>
@@ -1692,6 +1777,8 @@
       <c r="O14" s="19" t="n"/>
       <c r="P14" s="19" t="n"/>
       <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n"/>
@@ -1711,6 +1798,8 @@
       <c r="O15" s="19" t="n"/>
       <c r="P15" s="19" t="n"/>
       <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n"/>
@@ -1730,6 +1819,8 @@
       <c r="O16" s="19" t="n"/>
       <c r="P16" s="19" t="n"/>
       <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n"/>
@@ -1749,6 +1840,8 @@
       <c r="O17" s="19" t="n"/>
       <c r="P17" s="19" t="n"/>
       <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n"/>
@@ -1768,6 +1861,8 @@
       <c r="O18" s="19" t="n"/>
       <c r="P18" s="19" t="n"/>
       <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n"/>
@@ -1787,6 +1882,8 @@
       <c r="O19" s="19" t="n"/>
       <c r="P19" s="19" t="n"/>
       <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n"/>
@@ -1806,6 +1903,8 @@
       <c r="O20" s="19" t="n"/>
       <c r="P20" s="19" t="n"/>
       <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n"/>
@@ -1825,6 +1924,8 @@
       <c r="O21" s="19" t="n"/>
       <c r="P21" s="19" t="n"/>
       <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n"/>
@@ -1844,6 +1945,8 @@
       <c r="O22" s="19" t="n"/>
       <c r="P22" s="19" t="n"/>
       <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n"/>
@@ -1863,6 +1966,8 @@
       <c r="O23" s="19" t="n"/>
       <c r="P23" s="19" t="n"/>
       <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n"/>
@@ -1882,6 +1987,8 @@
       <c r="O24" s="19" t="n"/>
       <c r="P24" s="19" t="n"/>
       <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n"/>
@@ -1901,6 +2008,8 @@
       <c r="O25" s="19" t="n"/>
       <c r="P25" s="19" t="n"/>
       <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n"/>
@@ -1920,6 +2029,8 @@
       <c r="O26" s="19" t="n"/>
       <c r="P26" s="19" t="n"/>
       <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n"/>
@@ -1939,6 +2050,8 @@
       <c r="O27" s="19" t="n"/>
       <c r="P27" s="19" t="n"/>
       <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n"/>
@@ -1958,6 +2071,8 @@
       <c r="O28" s="19" t="n"/>
       <c r="P28" s="19" t="n"/>
       <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="n"/>
@@ -1977,6 +2092,8 @@
       <c r="O29" s="19" t="n"/>
       <c r="P29" s="19" t="n"/>
       <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n"/>
@@ -1996,6 +2113,8 @@
       <c r="O30" s="19" t="n"/>
       <c r="P30" s="19" t="n"/>
       <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="n"/>
@@ -2015,6 +2134,8 @@
       <c r="O31" s="19" t="n"/>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="19" t="n"/>
@@ -2034,6 +2155,8 @@
       <c r="O32" s="19" t="n"/>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="19" t="n"/>
@@ -2053,6 +2176,8 @@
       <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n"/>
@@ -2072,6 +2197,8 @@
       <c r="O34" s="19" t="n"/>
       <c r="P34" s="19" t="n"/>
       <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="n"/>
@@ -2091,6 +2218,8 @@
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="19" t="n"/>
       <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="19" t="n"/>
@@ -2110,6 +2239,8 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="n"/>
       <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -2129,6 +2260,8 @@
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="19" t="n"/>
@@ -2148,6 +2281,8 @@
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
       <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="19" t="n"/>
@@ -2167,6 +2302,8 @@
       <c r="O39" s="19" t="n"/>
       <c r="P39" s="19" t="n"/>
       <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="19" t="n"/>
@@ -2186,14 +2323,19 @@
       <c r="O40" s="19" t="n"/>
       <c r="P40" s="19" t="n"/>
       <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+      <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,lb"</formula1>
@@ -2228,7 +2370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2248,6 +2390,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2350,6 +2494,16 @@
           <t>Video</t>
         </is>
       </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Inclinación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -2419,6 +2573,8 @@
         </is>
       </c>
       <c r="Q4" s="12" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
+      <c r="S4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -2480,6 +2636,8 @@
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr"/>
+      <c r="R5" s="13" t="inlineStr"/>
+      <c r="S5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -2541,6 +2699,8 @@
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -2606,6 +2766,8 @@
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -2667,6 +2829,8 @@
         </is>
       </c>
       <c r="Q8" s="12" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
+      <c r="S8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="n"/>
@@ -2686,6 +2850,8 @@
       <c r="O9" s="19" t="n"/>
       <c r="P9" s="19" t="n"/>
       <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="n"/>
@@ -2705,6 +2871,8 @@
       <c r="O10" s="19" t="n"/>
       <c r="P10" s="19" t="n"/>
       <c r="Q10" s="19" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="n"/>
@@ -2724,6 +2892,8 @@
       <c r="O11" s="19" t="n"/>
       <c r="P11" s="19" t="n"/>
       <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n"/>
@@ -2743,6 +2913,8 @@
       <c r="O12" s="19" t="n"/>
       <c r="P12" s="19" t="n"/>
       <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n"/>
@@ -2762,6 +2934,8 @@
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
       <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n"/>
@@ -2781,6 +2955,8 @@
       <c r="O14" s="19" t="n"/>
       <c r="P14" s="19" t="n"/>
       <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n"/>
@@ -2800,6 +2976,8 @@
       <c r="O15" s="19" t="n"/>
       <c r="P15" s="19" t="n"/>
       <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n"/>
@@ -2819,6 +2997,8 @@
       <c r="O16" s="19" t="n"/>
       <c r="P16" s="19" t="n"/>
       <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n"/>
@@ -2838,6 +3018,8 @@
       <c r="O17" s="19" t="n"/>
       <c r="P17" s="19" t="n"/>
       <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n"/>
@@ -2857,6 +3039,8 @@
       <c r="O18" s="19" t="n"/>
       <c r="P18" s="19" t="n"/>
       <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n"/>
@@ -2876,6 +3060,8 @@
       <c r="O19" s="19" t="n"/>
       <c r="P19" s="19" t="n"/>
       <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n"/>
@@ -2895,6 +3081,8 @@
       <c r="O20" s="19" t="n"/>
       <c r="P20" s="19" t="n"/>
       <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n"/>
@@ -2914,6 +3102,8 @@
       <c r="O21" s="19" t="n"/>
       <c r="P21" s="19" t="n"/>
       <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n"/>
@@ -2933,6 +3123,8 @@
       <c r="O22" s="19" t="n"/>
       <c r="P22" s="19" t="n"/>
       <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n"/>
@@ -2952,6 +3144,8 @@
       <c r="O23" s="19" t="n"/>
       <c r="P23" s="19" t="n"/>
       <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n"/>
@@ -2971,6 +3165,8 @@
       <c r="O24" s="19" t="n"/>
       <c r="P24" s="19" t="n"/>
       <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n"/>
@@ -2990,6 +3186,8 @@
       <c r="O25" s="19" t="n"/>
       <c r="P25" s="19" t="n"/>
       <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n"/>
@@ -3009,6 +3207,8 @@
       <c r="O26" s="19" t="n"/>
       <c r="P26" s="19" t="n"/>
       <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n"/>
@@ -3028,6 +3228,8 @@
       <c r="O27" s="19" t="n"/>
       <c r="P27" s="19" t="n"/>
       <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n"/>
@@ -3047,6 +3249,8 @@
       <c r="O28" s="19" t="n"/>
       <c r="P28" s="19" t="n"/>
       <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="n"/>
@@ -3066,6 +3270,8 @@
       <c r="O29" s="19" t="n"/>
       <c r="P29" s="19" t="n"/>
       <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n"/>
@@ -3085,6 +3291,8 @@
       <c r="O30" s="19" t="n"/>
       <c r="P30" s="19" t="n"/>
       <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="n"/>
@@ -3104,6 +3312,8 @@
       <c r="O31" s="19" t="n"/>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="19" t="n"/>
@@ -3123,6 +3333,8 @@
       <c r="O32" s="19" t="n"/>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="19" t="n"/>
@@ -3142,6 +3354,8 @@
       <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n"/>
@@ -3161,6 +3375,8 @@
       <c r="O34" s="19" t="n"/>
       <c r="P34" s="19" t="n"/>
       <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="n"/>
@@ -3180,6 +3396,8 @@
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="19" t="n"/>
       <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="19" t="n"/>
@@ -3199,6 +3417,8 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="n"/>
       <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -3218,6 +3438,8 @@
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="19" t="n"/>
@@ -3237,6 +3459,8 @@
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
       <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="19" t="n"/>
@@ -3256,6 +3480,8 @@
       <c r="O39" s="19" t="n"/>
       <c r="P39" s="19" t="n"/>
       <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="19" t="n"/>
@@ -3275,14 +3501,19 @@
       <c r="O40" s="19" t="n"/>
       <c r="P40" s="19" t="n"/>
       <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+      <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,lb"</formula1>
@@ -3317,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3337,6 +3568,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3439,6 +3672,16 @@
           <t>Video</t>
         </is>
       </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Inclinación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -3500,6 +3743,8 @@
         </is>
       </c>
       <c r="Q4" s="12" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
+      <c r="S4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -3561,6 +3806,8 @@
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr"/>
+      <c r="R5" s="13" t="inlineStr"/>
+      <c r="S5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -3622,6 +3869,8 @@
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -3687,6 +3936,8 @@
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="n"/>
@@ -3706,6 +3957,8 @@
       <c r="O8" s="19" t="n"/>
       <c r="P8" s="19" t="n"/>
       <c r="Q8" s="19" t="n"/>
+      <c r="R8" s="19" t="n"/>
+      <c r="S8" s="19" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="n"/>
@@ -3725,6 +3978,8 @@
       <c r="O9" s="19" t="n"/>
       <c r="P9" s="19" t="n"/>
       <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="n"/>
@@ -3744,6 +3999,8 @@
       <c r="O10" s="19" t="n"/>
       <c r="P10" s="19" t="n"/>
       <c r="Q10" s="19" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="n"/>
@@ -3763,6 +4020,8 @@
       <c r="O11" s="19" t="n"/>
       <c r="P11" s="19" t="n"/>
       <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n"/>
@@ -3782,6 +4041,8 @@
       <c r="O12" s="19" t="n"/>
       <c r="P12" s="19" t="n"/>
       <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n"/>
@@ -3801,6 +4062,8 @@
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
       <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n"/>
@@ -3820,6 +4083,8 @@
       <c r="O14" s="19" t="n"/>
       <c r="P14" s="19" t="n"/>
       <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n"/>
@@ -3839,6 +4104,8 @@
       <c r="O15" s="19" t="n"/>
       <c r="P15" s="19" t="n"/>
       <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n"/>
@@ -3858,6 +4125,8 @@
       <c r="O16" s="19" t="n"/>
       <c r="P16" s="19" t="n"/>
       <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n"/>
@@ -3877,6 +4146,8 @@
       <c r="O17" s="19" t="n"/>
       <c r="P17" s="19" t="n"/>
       <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n"/>
@@ -3896,6 +4167,8 @@
       <c r="O18" s="19" t="n"/>
       <c r="P18" s="19" t="n"/>
       <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n"/>
@@ -3915,6 +4188,8 @@
       <c r="O19" s="19" t="n"/>
       <c r="P19" s="19" t="n"/>
       <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n"/>
@@ -3934,6 +4209,8 @@
       <c r="O20" s="19" t="n"/>
       <c r="P20" s="19" t="n"/>
       <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n"/>
@@ -3953,6 +4230,8 @@
       <c r="O21" s="19" t="n"/>
       <c r="P21" s="19" t="n"/>
       <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n"/>
@@ -3972,6 +4251,8 @@
       <c r="O22" s="19" t="n"/>
       <c r="P22" s="19" t="n"/>
       <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n"/>
@@ -3991,6 +4272,8 @@
       <c r="O23" s="19" t="n"/>
       <c r="P23" s="19" t="n"/>
       <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n"/>
@@ -4010,6 +4293,8 @@
       <c r="O24" s="19" t="n"/>
       <c r="P24" s="19" t="n"/>
       <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n"/>
@@ -4029,6 +4314,8 @@
       <c r="O25" s="19" t="n"/>
       <c r="P25" s="19" t="n"/>
       <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n"/>
@@ -4048,6 +4335,8 @@
       <c r="O26" s="19" t="n"/>
       <c r="P26" s="19" t="n"/>
       <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n"/>
@@ -4067,6 +4356,8 @@
       <c r="O27" s="19" t="n"/>
       <c r="P27" s="19" t="n"/>
       <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n"/>
@@ -4086,6 +4377,8 @@
       <c r="O28" s="19" t="n"/>
       <c r="P28" s="19" t="n"/>
       <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="n"/>
@@ -4105,6 +4398,8 @@
       <c r="O29" s="19" t="n"/>
       <c r="P29" s="19" t="n"/>
       <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n"/>
@@ -4124,6 +4419,8 @@
       <c r="O30" s="19" t="n"/>
       <c r="P30" s="19" t="n"/>
       <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="n"/>
@@ -4143,6 +4440,8 @@
       <c r="O31" s="19" t="n"/>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="19" t="n"/>
@@ -4162,6 +4461,8 @@
       <c r="O32" s="19" t="n"/>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="19" t="n"/>
@@ -4181,6 +4482,8 @@
       <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n"/>
@@ -4200,6 +4503,8 @@
       <c r="O34" s="19" t="n"/>
       <c r="P34" s="19" t="n"/>
       <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="n"/>
@@ -4219,6 +4524,8 @@
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="19" t="n"/>
       <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="19" t="n"/>
@@ -4238,6 +4545,8 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="n"/>
       <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -4257,6 +4566,8 @@
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="19" t="n"/>
@@ -4276,6 +4587,8 @@
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
       <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="19" t="n"/>
@@ -4295,6 +4608,8 @@
       <c r="O39" s="19" t="n"/>
       <c r="P39" s="19" t="n"/>
       <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="19" t="n"/>
@@ -4314,14 +4629,19 @@
       <c r="O40" s="19" t="n"/>
       <c r="P40" s="19" t="n"/>
       <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+      <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,lb"</formula1>
@@ -4356,7 +4676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4376,6 +4696,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4478,6 +4800,16 @@
           <t>Video</t>
         </is>
       </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Inclinación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -4539,6 +4871,8 @@
         </is>
       </c>
       <c r="Q4" s="12" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
+      <c r="S4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -4600,6 +4934,8 @@
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr"/>
+      <c r="R5" s="13" t="inlineStr"/>
+      <c r="S5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -4661,6 +4997,8 @@
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -4722,6 +5060,8 @@
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -4787,6 +5127,8 @@
         </is>
       </c>
       <c r="Q8" s="12" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
+      <c r="S8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="n"/>
@@ -4806,6 +5148,8 @@
       <c r="O9" s="19" t="n"/>
       <c r="P9" s="19" t="n"/>
       <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="n"/>
@@ -4825,6 +5169,8 @@
       <c r="O10" s="19" t="n"/>
       <c r="P10" s="19" t="n"/>
       <c r="Q10" s="19" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="n"/>
@@ -4844,6 +5190,8 @@
       <c r="O11" s="19" t="n"/>
       <c r="P11" s="19" t="n"/>
       <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n"/>
@@ -4863,6 +5211,8 @@
       <c r="O12" s="19" t="n"/>
       <c r="P12" s="19" t="n"/>
       <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n"/>
@@ -4882,6 +5232,8 @@
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
       <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n"/>
@@ -4901,6 +5253,8 @@
       <c r="O14" s="19" t="n"/>
       <c r="P14" s="19" t="n"/>
       <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n"/>
@@ -4920,6 +5274,8 @@
       <c r="O15" s="19" t="n"/>
       <c r="P15" s="19" t="n"/>
       <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n"/>
@@ -4939,6 +5295,8 @@
       <c r="O16" s="19" t="n"/>
       <c r="P16" s="19" t="n"/>
       <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n"/>
@@ -4958,6 +5316,8 @@
       <c r="O17" s="19" t="n"/>
       <c r="P17" s="19" t="n"/>
       <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n"/>
@@ -4977,6 +5337,8 @@
       <c r="O18" s="19" t="n"/>
       <c r="P18" s="19" t="n"/>
       <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n"/>
@@ -4996,6 +5358,8 @@
       <c r="O19" s="19" t="n"/>
       <c r="P19" s="19" t="n"/>
       <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n"/>
@@ -5015,6 +5379,8 @@
       <c r="O20" s="19" t="n"/>
       <c r="P20" s="19" t="n"/>
       <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n"/>
@@ -5034,6 +5400,8 @@
       <c r="O21" s="19" t="n"/>
       <c r="P21" s="19" t="n"/>
       <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n"/>
@@ -5053,6 +5421,8 @@
       <c r="O22" s="19" t="n"/>
       <c r="P22" s="19" t="n"/>
       <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n"/>
@@ -5072,6 +5442,8 @@
       <c r="O23" s="19" t="n"/>
       <c r="P23" s="19" t="n"/>
       <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n"/>
@@ -5091,6 +5463,8 @@
       <c r="O24" s="19" t="n"/>
       <c r="P24" s="19" t="n"/>
       <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n"/>
@@ -5110,6 +5484,8 @@
       <c r="O25" s="19" t="n"/>
       <c r="P25" s="19" t="n"/>
       <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n"/>
@@ -5129,6 +5505,8 @@
       <c r="O26" s="19" t="n"/>
       <c r="P26" s="19" t="n"/>
       <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n"/>
@@ -5148,6 +5526,8 @@
       <c r="O27" s="19" t="n"/>
       <c r="P27" s="19" t="n"/>
       <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n"/>
@@ -5167,6 +5547,8 @@
       <c r="O28" s="19" t="n"/>
       <c r="P28" s="19" t="n"/>
       <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="n"/>
@@ -5186,6 +5568,8 @@
       <c r="O29" s="19" t="n"/>
       <c r="P29" s="19" t="n"/>
       <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n"/>
@@ -5205,6 +5589,8 @@
       <c r="O30" s="19" t="n"/>
       <c r="P30" s="19" t="n"/>
       <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="n"/>
@@ -5224,6 +5610,8 @@
       <c r="O31" s="19" t="n"/>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="19" t="n"/>
@@ -5243,6 +5631,8 @@
       <c r="O32" s="19" t="n"/>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="19" t="n"/>
@@ -5262,6 +5652,8 @@
       <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n"/>
@@ -5281,6 +5673,8 @@
       <c r="O34" s="19" t="n"/>
       <c r="P34" s="19" t="n"/>
       <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="n"/>
@@ -5300,6 +5694,8 @@
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="19" t="n"/>
       <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="19" t="n"/>
@@ -5319,6 +5715,8 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="n"/>
       <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -5338,6 +5736,8 @@
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="19" t="n"/>
@@ -5357,6 +5757,8 @@
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
       <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="19" t="n"/>
@@ -5376,6 +5778,8 @@
       <c r="O39" s="19" t="n"/>
       <c r="P39" s="19" t="n"/>
       <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="19" t="n"/>
@@ -5395,14 +5799,19 @@
       <c r="O40" s="19" t="n"/>
       <c r="P40" s="19" t="n"/>
       <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+      <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,lb"</formula1>
@@ -5437,7 +5846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5457,6 +5866,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5559,6 +5970,16 @@
           <t>Video</t>
         </is>
       </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Máquina</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Inclinación</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -5620,6 +6041,8 @@
         </is>
       </c>
       <c r="Q4" s="12" t="inlineStr"/>
+      <c r="R4" s="13" t="inlineStr"/>
+      <c r="S4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -5681,6 +6104,8 @@
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr"/>
+      <c r="R5" s="13" t="inlineStr"/>
+      <c r="S5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -5742,6 +6167,8 @@
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -5803,6 +6230,8 @@
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -5874,6 +6303,8 @@
         </is>
       </c>
       <c r="Q8" s="12" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
+      <c r="S8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -5939,25 +6370,73 @@
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr"/>
+      <c r="R9" s="13" t="inlineStr"/>
+      <c r="S9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="19" t="n"/>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="19" t="n"/>
-      <c r="O10" s="19" t="n"/>
-      <c r="P10" s="19" t="n"/>
-      <c r="Q10" s="19" t="n"/>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Aeróbico</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr"/>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Aeróbico</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Bicicleta intervalos suaves</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>Z3</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr"/>
+      <c r="N10" s="13" t="inlineStr"/>
+      <c r="O10" s="13" t="inlineStr"/>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="inlineStr"/>
+      <c r="R10" s="13" t="inlineStr">
+        <is>
+          <t>Bicicleta</t>
+        </is>
+      </c>
+      <c r="S10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="n"/>
@@ -5977,6 +6456,8 @@
       <c r="O11" s="19" t="n"/>
       <c r="P11" s="19" t="n"/>
       <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n"/>
@@ -5996,6 +6477,8 @@
       <c r="O12" s="19" t="n"/>
       <c r="P12" s="19" t="n"/>
       <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n"/>
@@ -6015,6 +6498,8 @@
       <c r="O13" s="19" t="n"/>
       <c r="P13" s="19" t="n"/>
       <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n"/>
@@ -6034,6 +6519,8 @@
       <c r="O14" s="19" t="n"/>
       <c r="P14" s="19" t="n"/>
       <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n"/>
@@ -6053,6 +6540,8 @@
       <c r="O15" s="19" t="n"/>
       <c r="P15" s="19" t="n"/>
       <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n"/>
@@ -6072,6 +6561,8 @@
       <c r="O16" s="19" t="n"/>
       <c r="P16" s="19" t="n"/>
       <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n"/>
@@ -6091,6 +6582,8 @@
       <c r="O17" s="19" t="n"/>
       <c r="P17" s="19" t="n"/>
       <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n"/>
@@ -6110,6 +6603,8 @@
       <c r="O18" s="19" t="n"/>
       <c r="P18" s="19" t="n"/>
       <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n"/>
@@ -6129,6 +6624,8 @@
       <c r="O19" s="19" t="n"/>
       <c r="P19" s="19" t="n"/>
       <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n"/>
@@ -6148,6 +6645,8 @@
       <c r="O20" s="19" t="n"/>
       <c r="P20" s="19" t="n"/>
       <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="n"/>
@@ -6167,6 +6666,8 @@
       <c r="O21" s="19" t="n"/>
       <c r="P21" s="19" t="n"/>
       <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n"/>
@@ -6186,6 +6687,8 @@
       <c r="O22" s="19" t="n"/>
       <c r="P22" s="19" t="n"/>
       <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="19" t="n"/>
@@ -6205,6 +6708,8 @@
       <c r="O23" s="19" t="n"/>
       <c r="P23" s="19" t="n"/>
       <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n"/>
@@ -6224,6 +6729,8 @@
       <c r="O24" s="19" t="n"/>
       <c r="P24" s="19" t="n"/>
       <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="n"/>
@@ -6243,6 +6750,8 @@
       <c r="O25" s="19" t="n"/>
       <c r="P25" s="19" t="n"/>
       <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n"/>
@@ -6262,6 +6771,8 @@
       <c r="O26" s="19" t="n"/>
       <c r="P26" s="19" t="n"/>
       <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="19" t="n"/>
@@ -6281,6 +6792,8 @@
       <c r="O27" s="19" t="n"/>
       <c r="P27" s="19" t="n"/>
       <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n"/>
@@ -6300,6 +6813,8 @@
       <c r="O28" s="19" t="n"/>
       <c r="P28" s="19" t="n"/>
       <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="n"/>
@@ -6319,6 +6834,8 @@
       <c r="O29" s="19" t="n"/>
       <c r="P29" s="19" t="n"/>
       <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n"/>
@@ -6338,6 +6855,8 @@
       <c r="O30" s="19" t="n"/>
       <c r="P30" s="19" t="n"/>
       <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="19" t="n"/>
@@ -6357,6 +6876,8 @@
       <c r="O31" s="19" t="n"/>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="19" t="n"/>
@@ -6376,6 +6897,8 @@
       <c r="O32" s="19" t="n"/>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="19" t="n"/>
@@ -6395,6 +6918,8 @@
       <c r="O33" s="19" t="n"/>
       <c r="P33" s="19" t="n"/>
       <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n"/>
@@ -6414,6 +6939,8 @@
       <c r="O34" s="19" t="n"/>
       <c r="P34" s="19" t="n"/>
       <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="19" t="n"/>
@@ -6433,6 +6960,8 @@
       <c r="O35" s="19" t="n"/>
       <c r="P35" s="19" t="n"/>
       <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="19" t="n"/>
@@ -6452,6 +6981,8 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="n"/>
       <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="19" t="n"/>
@@ -6471,6 +7002,8 @@
       <c r="O37" s="19" t="n"/>
       <c r="P37" s="19" t="n"/>
       <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="19" t="n"/>
@@ -6490,6 +7023,8 @@
       <c r="O38" s="19" t="n"/>
       <c r="P38" s="19" t="n"/>
       <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="19" t="n"/>
@@ -6509,6 +7044,8 @@
       <c r="O39" s="19" t="n"/>
       <c r="P39" s="19" t="n"/>
       <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="19" t="n"/>
@@ -6528,14 +7065,19 @@
       <c r="O40" s="19" t="n"/>
       <c r="P40" s="19" t="n"/>
       <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="A4:A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rezagado,Principal,Complementario"</formula1>
+      <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset"</formula1>
+      <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="P4:P40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"kg,lb"</formula1>

</xml_diff>

<commit_message>
Bloque aeróbico: modalidad (con «Otro» manual), tiempo e intensidad por zona; botón para convertir
- Modalidad: Caminadora, Elíptica, Remadora, Escaladora, Air bike, Air ski, Aire libre,
  Natación u Otro (texto libre); inclinación solo en caminadora
- Botón «🏃 Aeróbico» en cada ejercicio: lo pasa a aeróbico y borra series, reps, RIR,
  tempo y descanso; «💪 Cambiar a fuerza» para regresar
- Excel: columna Modalidad

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EqTd92FjD8shfoXfrWiS9M
</commit_message>
<xml_diff>
--- a/plantilla-entrenamiento.xlsx
+++ b/plantilla-entrenamiento.xlsx
@@ -678,7 +678,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Aeróbico: pon Grupo = Aeróbico. En F1–F4 Series escribe los MINUTOS y en F1–F4 Reps la ZONA (Z1 a Z5). Llena Máquina e Inclinación (solo caminadora, en %). La FCE en pulsaciones se calcula sola con la edad y la FC en reposo del cliente.</t>
+          <t>Aeróbico: pon Grupo = Aeróbico. En F1–F4 Series escribe los MINUTOS y en F1–F4 Reps la ZONA (Z1 a Z5). Llena Modalidad (Caminadora, Elíptica, Remadora, Escaladora, Air bike, Air ski, Aire libre, Natación u otra que escribas) e Inclinación (solo caminadora, en %). La FCE en pulsaciones se calcula sola con la edad y la FC en reposo del cliente.</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Máquina</t>
+          <t>Modalidad</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
@@ -2332,7 +2332,7 @@
       <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
+      <formula1>"Caminadora,Elíptica,Remadora,Escaladora,Air bike,Air ski,Aire libre,Natación"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Máquina</t>
+          <t>Modalidad</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
@@ -3510,7 +3510,7 @@
       <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
+      <formula1>"Caminadora,Elíptica,Remadora,Escaladora,Air bike,Air ski,Aire libre,Natación"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
@@ -3674,7 +3674,7 @@
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Máquina</t>
+          <t>Modalidad</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
@@ -4638,7 +4638,7 @@
       <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
+      <formula1>"Caminadora,Elíptica,Remadora,Escaladora,Air bike,Air ski,Aire libre,Natación"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Máquina</t>
+          <t>Modalidad</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
@@ -5808,7 +5808,7 @@
       <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
+      <formula1>"Caminadora,Elíptica,Remadora,Escaladora,Air bike,Air ski,Aire libre,Natación"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>
@@ -5972,7 +5972,7 @@
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>Máquina</t>
+          <t>Modalidad</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Bicicleta intervalos suaves</t>
+          <t>Air bike intervalos suaves</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
@@ -6433,7 +6433,7 @@
       <c r="Q10" s="12" t="inlineStr"/>
       <c r="R10" s="13" t="inlineStr">
         <is>
-          <t>Bicicleta</t>
+          <t>Air bike</t>
         </is>
       </c>
       <c r="S10" s="13" t="inlineStr"/>
@@ -7074,7 +7074,7 @@
       <formula1>"Rezagado,Principal,Complementario,Aeróbico"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Caminadora,Bicicleta,Elíptica,Escaladora,Remo,Assault bike,Correr al aire libre,Otra"</formula1>
+      <formula1>"Caminadora,Elíptica,Remadora,Escaladora,Air bike,Air ski,Aire libre,Natación"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Aislado,Biserie,Triserie,Superserie,Megaserie,Dropset,Aeróbico"</formula1>

</xml_diff>